<commit_message>
fix(dcache): scrub remaining branch identifiers from prompts
</commit_message>
<xml_diff>
--- a/dcache_bug_prompts_v3.xlsx
+++ b/dcache_bug_prompts_v3.xlsx
@@ -514,7 +514,7 @@
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>green_base_bug_003 需要从空状态启动服务，red_base_bug_003 则要检查响应副本在调用方修改后的表现。一个分支在初始化成员表时直接崩溃，另一个分支在 Clone 后共享底层字节数组。请分别定位 nil map 写入和 slice ownership 失守的调用链，指出它们为什么跨越 cluster/protocol 层才暴露。先别改代码，帮我定位根因</t>
+          <t>对应缺陷分支 需要从空状态启动服务，对应缺陷分支 则要检查响应副本在调用方修改后的表现。一个分支在初始化成员表时直接崩溃，另一个分支在 Clone 后共享底层字节数组。请分别定位 nil map 写入和 slice ownership 失守的调用链，指出它们为什么跨越 cluster/protocol 层才暴露。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>对 green_base_bug_004 运行一个会取消的心跳上下文，对 red_base_bug_004 创建并关闭多个 Store，再查看 goroutine 和 ticker 数量。两种现象都表现为“调用方已经结束，后台工作仍在跑”，但触发点不同。请沿着 select 的退出分支、stop channel 和 ticker 清理路径定位根因，并给出不会依赖时序猜测的复现办法。先别改代码，帮我定位根因</t>
+          <t>对 对应缺陷分支 运行一个会取消的心跳上下文，对 对应缺陷分支 创建并关闭多个 Store，再查看 goroutine 和 ticker 数量。两种现象都表现为“调用方已经结束，后台工作仍在跑”，但触发点不同。请沿着 select 的退出分支、stop channel 和 ticker 清理路径定位根因，并给出不会依赖时序猜测的复现办法。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>在 green_base_bug_005 中让客户端连接一个未监听的地址，并验证调用方能否用 errors.Is/As 识别底层网络错误；在 red_base_bug_005 中请求 /api/status，服务不应因缺少 metrics 依赖而 panic。修正错误链和依赖装配，保证正常连接、正常状态接口和失败路径都保留清晰语义。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>在 对应缺陷分支 中让客户端连接一个未监听的地址，并验证调用方能否用 errors.Is/As 识别底层网络错误；在 对应缺陷分支 中请求 /api/status，服务不应因缺少 metrics 依赖而 panic。修正错误链和依赖装配，保证正常连接、正常状态接口和失败路径都保留清晰语义。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -567,7 +567,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>green_base_bug_006 的 DeletePrefix 在命中前缀时会卡在同一把 Store 锁上；red_base_bug_006 则在请求计数并发增长时调用 reset，`go test -race` 能看到非原子访问。请分别收窄锁的重入范围、恢复 Metrics 的原子读写，并确认清扫器、统计接口和删除操作可以同时运行。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>对应缺陷分支 的 DeletePrefix 在命中前缀时会卡在同一把 Store 锁上；对应缺陷分支 则在请求计数并发增长时调用 reset，`go test -race` 能看到非原子访问。请分别收窄锁的重入范围、恢复 Metrics 的原子读写，并确认清扫器、统计接口和删除操作可以同时运行。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -585,7 +585,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>先让同一地址的节点从 alive 变成 dead，再重新加入：green_base_bug_007 不应保留旧成员状态，Healthy 也不能只看地址；red_base_bug_007 的 Shutdown 不能因为额外增加 WaitGroup 计数而永久等待。修复成员更新和等待计数，保留现有节点 API，确保正常退出仍会等待真实会话。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>先让同一地址的节点从 alive 变成 dead，再重新加入：对应缺陷分支 不应保留旧成员状态，Healthy 也不能只看地址；对应缺陷分支 的 Shutdown 不能因为额外增加 WaitGroup 计数而永久等待。修复成员更新和等待计数，保留现有节点 API，确保正常退出仍会等待真实会话。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
@@ -603,7 +603,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>在 green_base_bug_008 中拿到缓存返回的 []byte 后修改它，再读取同一个 key，结果不能反过来改变 Store 内部值；red_base_bug_008 访问 /api/status 时依赖缺失应被安全处理，而不是由 nil 指针把 HTTP 服务打崩。请修复缓存数据的所有权边界和 Web 依赖注入，避免用全局状态掩盖问题。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>在 对应缺陷分支 中拿到缓存返回的 []byte 后修改它，再读取同一个 key，结果不能反过来改变 Store 内部值；对应缺陷分支 访问 /api/status 时依赖缺失应被安全处理，而不是由 nil 指针把 HTTP 服务打崩。请修复缓存数据的所有权边界和 Web 依赖注入，避免用全局状态掩盖问题。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>green_base_bug_009 对非法命令参数返回成功响应，客户端无法知道请求实际上没有执行；red_base_bug_009 的 TTL 在服务端编码和客户端解码之间被重复偏移，永久值与不存在值会混淆。请从 Validate、dispatch、Response.Extra 到 Client.TTL 的完整链路修复错误码和数值协议，覆盖正常 TTL、-1 和 -2 三种语义。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>对应缺陷分支 对非法命令参数返回成功响应，客户端无法知道请求实际上没有执行；对应缺陷分支 的 TTL 在服务端编码和客户端解码之间被重复偏移，永久值与不存在值会混淆。请从 Validate、dispatch、Response.Extra 到 Client.TTL 的完整链路修复错误码和数值协议，覆盖正常 TTL、-1 和 -2 三种语义。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
@@ -639,7 +639,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>green_base_bug_010 把连接超时配置强行变成无限期，空闲 TCP 会话因此长期占用 goroutine；red_base_bug_010 的 SnapshotItems 把内部 Value 直接带出，迁移方修改快照会污染缓存。修复连接生命周期和快照复制，确保关闭、超时、迁移读取都不会改变既有 API 行为。不要新增针对该缺陷的测试文件、注释或文档。</t>
+          <t>对应缺陷分支 把连接超时配置强行变成无限期，空闲 TCP 会话因此长期占用 goroutine；对应缺陷分支 的 SnapshotItems 把内部 Value 直接带出，迁移方修改快照会污染缓存。修复连接生命周期和快照复制，确保关闭、超时、迁移读取都不会改变既有 API 行为。不要新增针对该缺陷的测试文件、注释或文档。</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>

</xml_diff>